<commit_message>
[site] move model pages to top-level URLs — drop the /sim prefix entirely
The 8 model pages now live at clean root URLs (/trajectory, /forecasts, /fisc,
/unemployment, /references, /time-dividend, /sectors, /aggregate) instead of
/sim/X. Moved public/sim/{*.html,static,data} -> public/{*.html,static,data},
stripped every /sim ref in the HTML/JS, fixed the publish nav.js prefix + brand.
TopBar links + vercel updated: clean-URL rewrites for the 8 pages, SPA catch-all
excludes static/data, and old /sim/* links 301 to the new root paths. Source
(docs/ dev server) already used clean paths. Build verified; files serve at root,
/sim 404s. NOTE: bake_sim_static.py still emits /sim — needs updating before the
next re-bake (flagged for the code-cleanup pass).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/economy-model/mpc_spreadsheet/MPC Calc.xlsx
+++ b/docs/economy-model/mpc_spreadsheet/MPC Calc.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/17c67371d77ccfb8/Documents/Crypto/spice-dashboard/docs/economy-model/mpc_spreadsheet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="119" documentId="8_{0252EE9B-E084-4FE6-ACA0-6F1DC93FB747}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD5B2C0B-13AF-4941-9268-3A7DAAEF06A9}"/>
+  <xr:revisionPtr revIDLastSave="120" documentId="8_{0252EE9B-E084-4FE6-ACA0-6F1DC93FB747}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{320D290D-313B-4097-8600-57FD0E5F01B6}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="750" xr2:uid="{25826AAD-6613-48A6-9158-3D5A8725E2E6}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="750" activeTab="2" xr2:uid="{25826AAD-6613-48A6-9158-3D5A8725E2E6}"/>
   </bookViews>
   <sheets>
     <sheet name="TopSheet" sheetId="1" r:id="rId1"/>
     <sheet name="basket_trajectory" sheetId="8" state="hidden" r:id="rId2"/>
-    <sheet name="basket_composition" sheetId="7" state="hidden" r:id="rId3"/>
+    <sheet name="basket_composition" sheetId="7" r:id="rId3"/>
     <sheet name="maryfontaine_headlines" sheetId="2" state="hidden" r:id="rId4"/>
     <sheet name="external_by_sector (2)" sheetId="12" r:id="rId5"/>
     <sheet name="mpc_calc_per_company (2)" sheetId="11" r:id="rId6"/>

</xml_diff>